<commit_message>
removed v2g in dispatchable prod limit
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Base_KS_setup.xlsx
+++ b/SuppXLS/Scen_Base_KS_setup.xlsx
@@ -589,7 +589,7 @@
     <author>xli9</author>
   </authors>
   <commentList>
-    <comment ref="C4" authorId="0">
+    <comment ref="C5" authorId="0">
       <text>
         <r>
           <rPr>
@@ -2708,13 +2708,13 @@
     <t>Trd_bus_elc_134</t>
   </si>
   <si>
+    <t>Trd_car_elc_200</t>
+  </si>
+  <si>
+    <t>Trd_bus_elc_149</t>
+  </si>
+  <si>
     <t>~UC_T: UC_RHSRT~UP</t>
-  </si>
-  <si>
-    <t>Trd_car_elc_200</t>
-  </si>
-  <si>
-    <t>Trd_bus_elc_149</t>
   </si>
   <si>
     <t>~UC_T: UC_RHSRT~FX</t>
@@ -3559,11 +3559,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
@@ -3571,11 +3566,17 @@
     </font>
     <font>
       <b/>
+      <sz val="8"/>
+      <name val="Tahoma"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
@@ -3587,12 +3588,11 @@
     </font>
     <font>
       <b/>
-      <sz val="8"/>
+      <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
@@ -18285,9 +18285,6 @@
     <row r="4" ht="29" spans="1:34">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="7" t="s">
-        <v>658</v>
-      </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
@@ -18311,7 +18308,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="15"/>
       <c r="Z4" s="16" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="AA4" s="14">
         <v>36</v>
@@ -18321,7 +18318,7 @@
         <v>-36</v>
       </c>
       <c r="AF4" s="14" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AG4" s="14">
         <v>149</v>
@@ -18334,6 +18331,9 @@
     <row r="5" ht="29" spans="1:34">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>660</v>
+      </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -18671,7 +18671,7 @@
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="10" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
@@ -18688,7 +18688,7 @@
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
       <c r="T10" s="10" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="U10" s="15"/>
       <c r="V10" s="15"/>
@@ -19675,7 +19675,7 @@
       <c r="X28" s="15"/>
       <c r="Y28" s="15"/>
       <c r="Z28" s="16" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AA28" s="14">
         <v>149</v>
@@ -19925,7 +19925,7 @@
       <c r="R34" s="7"/>
       <c r="S34" s="7"/>
       <c r="T34" s="10" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="U34" s="15"/>
       <c r="V34" s="15"/>
@@ -21661,7 +21661,7 @@
       <c r="A3" s="5"/>
       <c r="B3" s="6"/>
       <c r="C3" s="7" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
@@ -21805,7 +21805,7 @@
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="10" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="J10" s="5"/>
       <c r="L10" s="5"/>

</xml_diff>